<commit_message>
refresh tracker, prepare move on ideation polish
</commit_message>
<xml_diff>
--- a/01_planning/2_PwC_6Week_Tracker.xlsx
+++ b/01_planning/2_PwC_6Week_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ez_us/Documents/Deaf_life_plan/Portofilo/Google_UX_design/NF2_case/01_planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C56CB6-E810-DE4A-9FE7-F8F362898A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E167FDA1-F912-824B-B4F3-3E9B5AB5BFDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="40960" windowHeight="23040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4100" yWindow="600" windowWidth="22940" windowHeight="16960" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracker" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="127">
   <si>
     <t>Week</t>
   </si>
@@ -409,6 +409,15 @@
   </si>
   <si>
     <t>How to use: update Status (dropdown) on Tracker. Owner colors: blue=Echo, green=Yiran, gold=Shengxuan, purple=All. Source: 01_planning/2_PwC_6Week_Plan.md</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Dropped</t>
+  </si>
+  <si>
+    <t>In progress</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1053,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>15</v>
+        <v>124</v>
       </c>
       <c r="I2" s="2"/>
     </row>
@@ -1071,7 +1080,7 @@
         <v>19</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>15</v>
+        <v>124</v>
       </c>
       <c r="I3" s="2"/>
     </row>
@@ -1098,7 +1107,7 @@
         <v>23</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>15</v>
+        <v>125</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1125,7 +1134,7 @@
         <v>26</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>15</v>
+        <v>126</v>
       </c>
       <c r="I5" s="2"/>
     </row>
@@ -1891,7 +1900,7 @@
       </c>
       <c r="B13" s="5" t="str">
         <f>COUNTIF(Tracker!H:H,"Done")&amp;" / "&amp;(COUNTA(Tracker!D:D)-1)</f>
-        <v>0 / 28</v>
+        <v>2 / 28</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
add crazy 8 canvas and reedit the plan -assignment compititor audit
</commit_message>
<xml_diff>
--- a/01_planning/2_PwC_6Week_Tracker.xlsx
+++ b/01_planning/2_PwC_6Week_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ez_us/Documents/Deaf_life_plan/Portofilo/Google_UX_design/NF2_case/01_planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E167FDA1-F912-824B-B4F3-3E9B5AB5BFDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7211612-FACA-3945-BF99-B13D219078A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4100" yWindow="600" windowWidth="22940" windowHeight="16960" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10800" yWindow="5600" windowWidth="22940" windowHeight="16960" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracker" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="128">
   <si>
     <t>Week</t>
   </si>
@@ -159,18 +159,12 @@
     <t>2.1</t>
   </si>
   <si>
-    <t>HMW statements (5) + Crazy Eights workshop</t>
-  </si>
-  <si>
     <t>HMW list + sketches</t>
   </si>
   <si>
     <t>2.2</t>
   </si>
   <si>
-    <t>User flow: Log Event -&gt; Timeline -&gt; Summary</t>
-  </si>
-  <si>
     <t>Flowchart</t>
   </si>
   <si>
@@ -195,12 +189,6 @@
     <t>2.5</t>
   </si>
   <si>
-    <t>Accessibility heuristic pass on lo-fi</t>
-  </si>
-  <si>
-    <t>Issue list</t>
-  </si>
-  <si>
     <t>Aug 3-9</t>
   </si>
   <si>
@@ -418,6 +406,21 @@
   </si>
   <si>
     <t>In progress</t>
+  </si>
+  <si>
+    <t>w3</t>
+  </si>
+  <si>
+    <t>Goal Statements + Crazy Eights workshop</t>
+  </si>
+  <si>
+    <t>IA + User flow: Log Event -&gt; Timeline -&gt; Summary</t>
+  </si>
+  <si>
+    <t>Competitor Audit</t>
+  </si>
+  <si>
+    <t>Sheet</t>
   </si>
 </sst>
 </file>
@@ -437,62 +440,63 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF2E74B5"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF7030A0"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF548235"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFBF8F00"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -644,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -722,6 +726,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1053,7 +1060,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="I2" s="2"/>
     </row>
@@ -1080,7 +1087,7 @@
         <v>19</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="I3" s="2"/>
     </row>
@@ -1107,7 +1114,7 @@
         <v>23</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1134,7 +1141,7 @@
         <v>26</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="I5" s="2"/>
     </row>
@@ -1161,7 +1168,7 @@
         <v>30</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>15</v>
+        <v>121</v>
       </c>
       <c r="I6" s="2"/>
     </row>
@@ -1188,7 +1195,7 @@
         <v>33</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>15</v>
+        <v>122</v>
       </c>
       <c r="I7" s="2"/>
     </row>
@@ -1215,9 +1222,11 @@
         <v>36</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" s="11"/>
+        <v>120</v>
+      </c>
+      <c r="I8" s="32" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="20" x14ac:dyDescent="0.2">
       <c r="A9" s="25">
@@ -1233,16 +1242,16 @@
         <v>39</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>40</v>
+        <v>124</v>
       </c>
       <c r="F9" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -1257,19 +1266,19 @@
         <v>38</v>
       </c>
       <c r="D10" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="15" t="s">
-        <v>44</v>
-      </c>
       <c r="H10" s="15" t="s">
-        <v>15</v>
+        <v>122</v>
       </c>
       <c r="I10" s="2"/>
     </row>
@@ -1284,16 +1293,16 @@
         <v>38</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H11" s="15" t="s">
         <v>15</v>
@@ -1311,16 +1320,16 @@
         <v>38</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F12" s="20" t="s">
         <v>29</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>15</v>
@@ -1338,16 +1347,16 @@
         <v>38</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>52</v>
+        <v>126</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>22</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>53</v>
+        <v>127</v>
       </c>
       <c r="H13" s="15" t="s">
         <v>15</v>
@@ -1359,22 +1368,22 @@
         <v>3</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>15</v>
@@ -1386,22 +1395,22 @@
         <v>3</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C15" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="16" t="s">
-        <v>59</v>
-      </c>
       <c r="E15" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F15" s="19" t="s">
         <v>22</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>15</v>
@@ -1413,22 +1422,22 @@
         <v>3</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F16" s="28" t="s">
         <v>22</v>
       </c>
       <c r="G16" s="22" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="H16" s="22" t="s">
         <v>15</v>
@@ -1440,22 +1449,22 @@
         <v>3</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F17" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>15</v>
@@ -1467,22 +1476,22 @@
         <v>3</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F18" s="20" t="s">
         <v>29</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>15</v>
@@ -1494,22 +1503,22 @@
         <v>4</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>15</v>
@@ -1521,22 +1530,22 @@
         <v>4</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C20" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="D20" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="D20" s="16" t="s">
-        <v>76</v>
-      </c>
       <c r="E20" s="15" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F20" s="20" t="s">
         <v>29</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>15</v>
@@ -1548,22 +1557,22 @@
         <v>4</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F21" s="19" t="s">
         <v>22</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>15</v>
@@ -1575,22 +1584,22 @@
         <v>4</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F22" s="19" t="s">
         <v>22</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>15</v>
@@ -1602,22 +1611,22 @@
         <v>5</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F23" s="20" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H23" s="15" t="s">
         <v>15</v>
@@ -1629,22 +1638,22 @@
         <v>5</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C24" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D24" s="16" t="s">
-        <v>90</v>
-      </c>
       <c r="E24" s="15" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F24" s="19" t="s">
         <v>22</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>15</v>
@@ -1656,22 +1665,22 @@
         <v>5</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F25" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="H25" s="15" t="s">
         <v>15</v>
@@ -1683,22 +1692,22 @@
         <v>6</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F26" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H26" s="15" t="s">
         <v>15</v>
@@ -1710,22 +1719,22 @@
         <v>6</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C27" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="D27" s="16" t="s">
-        <v>101</v>
-      </c>
       <c r="E27" s="15" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F27" s="19" t="s">
         <v>22</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>15</v>
@@ -1737,22 +1746,22 @@
         <v>6</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F28" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>15</v>
@@ -1764,22 +1773,22 @@
         <v>6</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F29" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H29" s="15" t="s">
         <v>15</v>
@@ -1809,52 +1818,52 @@
   <sheetData>
     <row r="1" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B8" s="5"/>
     </row>
@@ -1864,7 +1873,7 @@
       </c>
       <c r="B9" s="5">
         <f>COUNTIF(Tracker!F:F,"Echo")</f>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1882,7 +1891,7 @@
       </c>
       <c r="B11" s="5">
         <f>COUNTIF(Tracker!F:F,"Shengxuan")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1896,16 +1905,16 @@
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B13" s="5" t="str">
         <f>COUNTIF(Tracker!H:H,"Done")&amp;" / "&amp;(COUNTA(Tracker!D:D)-1)</f>
-        <v>2 / 28</v>
+        <v>5 / 28</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update planning and design files
</commit_message>
<xml_diff>
--- a/01_planning/2_PwC_6Week_Tracker.xlsx
+++ b/01_planning/2_PwC_6Week_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ez_us/Documents/Deaf_life_plan/Portofilo/Google_UX_design/NF2_case/01_planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7211612-FACA-3945-BF99-B13D219078A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CC318BA-6449-F04C-99B2-3D21C99C060D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10800" yWindow="5600" windowWidth="22940" windowHeight="16960" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10800" yWindow="4640" windowWidth="22940" windowHeight="16960" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracker" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracker!$A$1:$I$29</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1359,7 +1359,7 @@
         <v>127</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="B13" s="5" t="str">
         <f>COUNTIF(Tracker!H:H,"Done")&amp;" / "&amp;(COUNTA(Tracker!D:D)-1)</f>
-        <v>5 / 28</v>
+        <v>6 / 28</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
use the case apply eihub, update the 6 week, plan; build the accessibility check list
</commit_message>
<xml_diff>
--- a/01_planning/2_PwC_6Week_Tracker.xlsx
+++ b/01_planning/2_PwC_6Week_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ez_us/Documents/Deaf_life_plan/Portofilo/Google_UX_design/NF2_case/01_planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CC318BA-6449-F04C-99B2-3D21C99C060D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F498467-CCF1-964D-BC9D-FCA5F049B2D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10800" yWindow="4640" windowWidth="22940" windowHeight="16960" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="129">
   <si>
     <t>Week</t>
   </si>
@@ -249,9 +249,6 @@
     <t>4.1</t>
   </si>
   <si>
-    <t>Remaining 3 hi-fi screens + clickable prototype</t>
-  </si>
-  <si>
     <t>Figma prototype link</t>
   </si>
   <si>
@@ -421,6 +418,12 @@
   </si>
   <si>
     <t>Sheet</t>
+  </si>
+  <si>
+    <t>Blocked</t>
+  </si>
+  <si>
+    <t>Remaining several hi-fi screens + clickable prototype</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1063,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I2" s="2"/>
     </row>
@@ -1087,7 +1090,7 @@
         <v>19</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I3" s="2"/>
     </row>
@@ -1114,7 +1117,7 @@
         <v>23</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1141,7 +1144,7 @@
         <v>26</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I5" s="2"/>
     </row>
@@ -1168,7 +1171,7 @@
         <v>30</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I6" s="2"/>
     </row>
@@ -1195,7 +1198,7 @@
         <v>33</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I7" s="2"/>
     </row>
@@ -1222,10 +1225,10 @@
         <v>36</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I8" s="32" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="20" x14ac:dyDescent="0.2">
@@ -1242,7 +1245,7 @@
         <v>39</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F9" s="18" t="s">
         <v>18</v>
@@ -1251,7 +1254,7 @@
         <v>40</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -1269,7 +1272,7 @@
         <v>41</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F10" s="20" t="s">
         <v>29</v>
@@ -1278,7 +1281,7 @@
         <v>42</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I10" s="2"/>
     </row>
@@ -1350,16 +1353,16 @@
         <v>49</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>22</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -1386,7 +1389,7 @@
         <v>54</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>15</v>
+        <v>121</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -1413,7 +1416,7 @@
         <v>57</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="I15" s="2"/>
     </row>
@@ -1440,7 +1443,7 @@
         <v>60</v>
       </c>
       <c r="H16" s="22" t="s">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="I16" s="11"/>
     </row>
@@ -1467,7 +1470,7 @@
         <v>63</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="I17" s="2"/>
     </row>
@@ -1494,7 +1497,7 @@
         <v>66</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
       <c r="I18" s="2"/>
     </row>
@@ -1512,16 +1515,16 @@
         <v>69</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>15</v>
+        <v>121</v>
       </c>
       <c r="I19" s="2"/>
     </row>
@@ -1536,19 +1539,19 @@
         <v>68</v>
       </c>
       <c r="D20" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="E20" s="15" t="s">
         <v>72</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>73</v>
       </c>
       <c r="F20" s="20" t="s">
         <v>29</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="I20" s="2"/>
     </row>
@@ -1563,16 +1566,16 @@
         <v>68</v>
       </c>
       <c r="D21" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="E21" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="F21" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="15" t="s">
         <v>76</v>
-      </c>
-      <c r="F21" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>77</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>15</v>
@@ -1590,19 +1593,19 @@
         <v>68</v>
       </c>
       <c r="D22" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E22" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="F22" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="F22" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="G22" s="15" t="s">
-        <v>80</v>
-      </c>
       <c r="H22" s="15" t="s">
-        <v>15</v>
+        <v>121</v>
       </c>
       <c r="I22" s="2"/>
     </row>
@@ -1611,22 +1614,22 @@
         <v>5</v>
       </c>
       <c r="B23" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="D23" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="E23" s="15" t="s">
         <v>83</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>84</v>
       </c>
       <c r="F23" s="20" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H23" s="15" t="s">
         <v>15</v>
@@ -1638,22 +1641,22 @@
         <v>5</v>
       </c>
       <c r="B24" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C24" s="15" t="s">
-        <v>82</v>
-      </c>
       <c r="D24" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="E24" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="F24" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="15" t="s">
         <v>87</v>
-      </c>
-      <c r="F24" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="G24" s="15" t="s">
-        <v>88</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>15</v>
@@ -1665,22 +1668,22 @@
         <v>5</v>
       </c>
       <c r="B25" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C25" s="15" t="s">
-        <v>82</v>
-      </c>
       <c r="D25" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E25" s="15" t="s">
         <v>89</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>90</v>
       </c>
       <c r="F25" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H25" s="15" t="s">
         <v>15</v>
@@ -1692,22 +1695,22 @@
         <v>6</v>
       </c>
       <c r="B26" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="D26" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="D26" s="16" t="s">
+      <c r="E26" s="15" t="s">
         <v>94</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>95</v>
       </c>
       <c r="F26" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H26" s="15" t="s">
         <v>15</v>
@@ -1719,22 +1722,22 @@
         <v>6</v>
       </c>
       <c r="B27" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C27" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="C27" s="15" t="s">
-        <v>93</v>
-      </c>
       <c r="D27" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E27" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="F27" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="G27" s="15" t="s">
         <v>98</v>
-      </c>
-      <c r="F27" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>99</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>15</v>
@@ -1746,22 +1749,22 @@
         <v>6</v>
       </c>
       <c r="B28" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="C28" s="15" t="s">
-        <v>93</v>
-      </c>
       <c r="D28" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E28" s="15" t="s">
         <v>100</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>101</v>
       </c>
       <c r="F28" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>15</v>
@@ -1773,22 +1776,22 @@
         <v>6</v>
       </c>
       <c r="B29" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="C29" s="15" t="s">
-        <v>93</v>
-      </c>
       <c r="D29" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="E29" s="15" t="s">
         <v>103</v>
-      </c>
-      <c r="E29" s="15" t="s">
-        <v>104</v>
       </c>
       <c r="F29" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H29" s="15" t="s">
         <v>15</v>
@@ -1818,52 +1821,52 @@
   <sheetData>
     <row r="1" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>107</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>111</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B8" s="5"/>
     </row>
@@ -1873,7 +1876,7 @@
       </c>
       <c r="B9" s="5">
         <f>COUNTIF(Tracker!F:F,"Echo")</f>
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1882,7 +1885,7 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Tracker!F:F,"Yiran")</f>
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1891,7 +1894,7 @@
       </c>
       <c r="B11" s="5">
         <f>COUNTIF(Tracker!F:F,"Shengxuan")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1905,16 +1908,16 @@
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B13" s="5" t="str">
         <f>COUNTIF(Tracker!H:H,"Done")&amp;" / "&amp;(COUNTA(Tracker!D:D)-1)</f>
-        <v>6 / 28</v>
+        <v>10 / 28</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>